<commit_message>
fix: jump to/from pacman #2
</commit_message>
<xml_diff>
--- a/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/第一章.xlsx
+++ b/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/第一章.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12080"/>
+    <workbookView windowWidth="24750" windowHeight="12790"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="79">
   <si>
     <t>ID</t>
   </si>
@@ -809,6 +809,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>挑战的话Boy待会自然会知道</t>
     </r>
     <r>
@@ -2629,13 +2635,16 @@
       <c r="B33" t="s">
         <v>12</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="K33" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="2">
         <v>1032</v>
+      </c>
+      <c r="B34" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:12">

</xml_diff>

<commit_message>
fix: multiple Pacman un-jump-able
</commit_message>
<xml_diff>
--- a/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/第一章.xlsx
+++ b/gal/Assets/Resources/VNovelizerRes/ExcelVNScripts/第一章.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12080"/>
+    <workbookView windowWidth="24750" windowHeight="12790"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -447,6 +447,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>谁会这么做啊</t>
     </r>
     <r>

</xml_diff>